<commit_message>
Calculadora (Excel): dominio .com, correo vigente, Alicante, WhatsApp 689 y tarifa Junior 1.200 €
El Excel que se descarga el lead decía globaltalentconnections.es, info@internationalgtc.es
(buzón que ya no existe), «presencia en Miami» y WhatsApp +34 622 85 04 23. La tarifa Junior
era 1.100 €/mes, por debajo del precio mínimo de 1.200. Solo se tocan las cadenas y esa
constante de la fórmula; el resto del libro queda intacto.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Calculadora-de-Ahorro-Estrategico-GTC.xlsx
+++ b/public/Calculadora-de-Ahorro-Estrategico-GTC.xlsx
@@ -32,7 +32,7 @@
     <t>📖  Guía de Uso — Calculadora de Ahorro GTC</t>
   </si>
   <si>
-    <t>Global Talent Connections · www.globaltalentconnections.es</t>
+    <t>Global Talent Connections · www.globaltalent-connections.com</t>
   </si>
   <si>
     <t xml:space="preserve">  🟦  CÓMO USAR ESTA CALCULADORA</t>
@@ -86,13 +86,13 @@
     <t xml:space="preserve">  📞  ¿TIENES DUDAS?</t>
   </si>
   <si>
-    <t xml:space="preserve">  🌐  www.globaltalentconnections.es</t>
+    <t xml:space="preserve">  🌐  www.globaltalent-connections.com</t>
   </si>
   <si>
-    <t xml:space="preserve">  📧 info@internationalgtc.es</t>
+    <t xml:space="preserve">  📧 info@globaltalent-connections.com</t>
   </si>
   <si>
-    <t xml:space="preserve">  📍  Con presencia en Miami</t>
+    <t xml:space="preserve">  📍  Alicante, España</t>
   </si>
   <si>
     <t xml:space="preserve">💼  Calculadora de Ahorro 
@@ -261,7 +261,7 @@
     <t>ℹ  El ahorro comienza desde la primera nómina</t>
   </si>
   <si>
-    <t xml:space="preserve">  Resultados en base a los datos introducidos en la hoja 🧮 Calculadora  ·  globaltalentconnections.es</t>
+    <t xml:space="preserve">  Resultados en base a los datos introducidos en la hoja 🧮 Calculadora  ·  globaltalent-connections.com</t>
   </si>
   <si>
     <t xml:space="preserve">  🎯  CONCLUSIÓN PERSONALIZADA</t>
@@ -270,7 +270,7 @@
     <t xml:space="preserve">  ¿Listo para dar el siguiente paso? Escríbenos y revisemos juntos los perfiles que tu empresa necesita.</t>
   </si>
   <si>
-    <t xml:space="preserve">  🌐www.globaltalentconnections.es/    |    📧  info@internationalgtc.es    |    💬  WhatsApp: +34 622 85 04 23</t>
+    <t xml:space="preserve">  🌐www.globaltalent-connections.com/    |    📧  info@globaltalent-connections.com    |    💬  WhatsApp: +34 689 53 98 96</t>
   </si>
 </sst>
 </file>
@@ -3514,7 +3514,7 @@
       </c>
       <c r="E15" s="51"/>
       <c r="F15" s="56">
-        <f>IF(C11="Junior",1100*12,IF(C11="Mid",1400*12,IF(C11="Senior",1650*12,0)))</f>
+        <f>IF(C11="Junior",1200*12,IF(C11="Mid",1400*12,IF(C11="Senior",1650*12,0)))</f>
         <v>19800</v>
       </c>
       <c r="G15" s="57">

</xml_diff>